<commit_message>
Remove Eleduck and update catalog to 73 entries
</commit_message>
<xml_diff>
--- a/platform-catalog.xlsx
+++ b/platform-catalog.xlsx
@@ -2,11 +2,11 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一覧" sheetId="1" r:id="R02dbab62412e4966"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="詳細情報" sheetId="2" r:id="R930b571a656849bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="関連事例・サービス" sheetId="3" r:id="R70f8ddea37d74621"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="横断比較・方針" sheetId="4" r:id="R9d31ef2882ac44c3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レビュー・出典" sheetId="5" r:id="Re92aedc193894906"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="一覧" sheetId="1" r:id="Redf26d7955764bb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="詳細情報" sheetId="2" r:id="R02936b05e7f84ae5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="関連事例・サービス" sheetId="3" r:id="R20cc33f821d24630"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="横断比較・方針" sheetId="4" r:id="R7b3225d5d5084c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="レビュー・出典" sheetId="5" r:id="R1269e5bfbaa541e6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -103,7 +103,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="25">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -155,6 +155,12 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="right" vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -163,8 +169,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PlatformIndex" displayName="PlatformIndex" ref="A5:S79" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:S79"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="6" name="PlatformIndex" displayName="PlatformIndex" ref="A5:S78" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:S78"/>
   <x:tableColumns count="19">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="サイト・コミュニティ名"/>
@@ -191,8 +197,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PlatformDetails" displayName="PlatformDetails" ref="A5:F141" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
-  <x:autoFilter ref="A5:F141"/>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="7" name="PlatformDetails" displayName="PlatformDetails" ref="A5:F139" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:autoFilter ref="A5:F139"/>
   <x:tableColumns count="6">
     <x:tableColumn id="1" name="ID"/>
     <x:tableColumn id="2" name="サイト・コミュニティ名"/>
@@ -486,7 +492,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
-        <x:v>本文・比較表から抽出した74項目。サイト内コミュニティを含む。R1/R2は「レビュー・出典」を参照。</x:v>
+        <x:v>本文・比較表から抽出後、ユーザー指定の1項目を除外した73項目。サイト内コミュニティを含む。R1/R2は「レビュー・出典」を参照。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -3966,749 +3972,715 @@
       </x:c>
     </x:row>
     <x:row r="67" ht="60" customHeight="1">
-      <x:c r="A67" s="12" t="str">
-        <x:v>P62</x:v>
-      </x:c>
-      <x:c r="B67" s="12" t="str">
-        <x:v>電鴨社区</x:v>
-      </x:c>
-      <x:c r="C67" s="12" t="str">
-        <x:v>リモートワーク・製品公開</x:v>
-      </x:c>
-      <x:c r="D67" s="12" t="str">
+      <x:c r="A67" s="11" t="str">
+        <x:v>P63</x:v>
+      </x:c>
+      <x:c r="B67" s="11" t="str">
+        <x:v>CSDN</x:v>
+      </x:c>
+      <x:c r="C67" s="11" t="str">
+        <x:v>技術記事・ブログ</x:v>
+      </x:c>
+      <x:c r="D67" s="11" t="str">
         <x:v>中国</x:v>
       </x:c>
-      <x:c r="E67" s="12" t="str">
-        <x:v>働き方の交流から独立製品公開へ広がる。</x:v>
-      </x:c>
-      <x:c r="F67" s="12" t="str">
-        <x:v>Eleduck / 发布独立产品</x:v>
-      </x:c>
-      <x:c r="G67" s="12" t="str">
+      <x:c r="E67" s="11" t="str">
+        <x:v>中国語技術ブログと備忘録の蓄積。</x:v>
+      </x:c>
+      <x:c r="F67" s="11"/>
+      <x:c r="G67" s="11" t="str">
         <x:v>R2</x:v>
       </x:c>
-      <x:c r="H67" s="12" t="str">
+      <x:c r="H67" s="11" t="str">
         <x:v>原文記載なし</x:v>
       </x:c>
-      <x:c r="I67" s="18" t="str">
+      <x:c r="I67" s="11" t="str">
+        <x:v>登録会員</x:v>
+      </x:c>
+      <x:c r="J67" s="16" t="n">
+        <x:v>48000000</x:v>
+      </x:c>
+      <x:c r="K67" s="11" t="str">
+        <x:v>超・人</x:v>
+      </x:c>
+      <x:c r="L67" s="11" t="str">
+        <x:v>MAU/DAUは未確認</x:v>
+      </x:c>
+      <x:c r="M67" s="11" t="str">
+        <x:v>年平均新規利用者700万人、企業顧客・パートナー1,000社以上</x:v>
+      </x:c>
+      <x:c r="N67" s="11" t="str">
+        <x:v>掲載時点不明・2026-10-21確認</x:v>
+      </x:c>
+      <x:c r="O67" s="11" t="str">
+        <x:v>公式確認</x:v>
+      </x:c>
+      <x:c r="P67" s="11" t="str">
+        <x:v>https://www.csdn.net/company/index.html</x:v>
+      </x:c>
+      <x:c r="Q67" s="11" t="str">
+        <x:v>定量的な人数記載なし</x:v>
+      </x:c>
+      <x:c r="R67" s="11" t="str">
+        <x:v>公式会社案内の4,800万人超。ユーザー投稿にある5,100万人等を公式値と混同しない。</x:v>
+      </x:c>
+      <x:c r="S67" s="17" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="68" ht="60" customHeight="1">
+      <x:c r="A68" s="12" t="str">
+        <x:v>P64</x:v>
+      </x:c>
+      <x:c r="B68" s="12" t="str">
+        <x:v>Developpez.com</x:v>
+      </x:c>
+      <x:c r="C68" s="12" t="str">
+        <x:v>技術記事・Q&amp;A・学習</x:v>
+      </x:c>
+      <x:c r="D68" s="12" t="str">
+        <x:v>フランス語圏</x:v>
+      </x:c>
+      <x:c r="E68" s="12" t="str">
+        <x:v>ボランティアが運営する老舗の技術情報共有。</x:v>
+      </x:c>
+      <x:c r="F68" s="12" t="str">
+        <x:v>Le Club des Développeurs et IT Pro</x:v>
+      </x:c>
+      <x:c r="G68" s="12" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H68" s="12" t="str">
+        <x:v>https://developpez.com/</x:v>
+      </x:c>
+      <x:c r="I68" s="12" t="str">
+        <x:v>会員数（歴史値）</x:v>
+      </x:c>
+      <x:c r="J68" s="23" t="n">
+        <x:v>750000</x:v>
+      </x:c>
+      <x:c r="K68" s="12" t="str">
+        <x:v>人</x:v>
+      </x:c>
+      <x:c r="L68" s="12" t="str">
+        <x:v>月間最大400万UV・1,200万PV（歴史値）</x:v>
+      </x:c>
+      <x:c r="M68" s="12" t="str">
+        <x:v>2,000フォーラム、最大5,000投稿/日（同じ公表）</x:v>
+      </x:c>
+      <x:c r="N68" s="12" t="str">
+        <x:v>2017年公表記事・現在値は未確認</x:v>
+      </x:c>
+      <x:c r="O68" s="12" t="str">
+        <x:v>公式運営投稿・歴史値</x:v>
+      </x:c>
+      <x:c r="P68" s="12" t="str">
+        <x:v>https://www.developpez.net/forums/i1675688/club-professionnels-informatique/actualites/croissance-annuelle-16-reseau-social-club-developpez-com/</x:v>
+      </x:c>
+      <x:c r="Q68" s="12" t="str">
+        <x:v>月間最大400万UU・5,000投稿/日・14,000記事</x:v>
+      </x:c>
+      <x:c r="R68" s="12" t="str">
+        <x:v>原レポートの月間400万UUには古い公表と一致する値が含まれる。2026年の実測値とは扱わない。</x:v>
+      </x:c>
+      <x:c r="S68" s="24" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="69" ht="60" customHeight="1">
+      <x:c r="A69" s="11" t="str">
+        <x:v>P65</x:v>
+      </x:c>
+      <x:c r="B69" s="11" t="str">
+        <x:v>Zeste de Savoir</x:v>
+      </x:c>
+      <x:c r="C69" s="11" t="str">
+        <x:v>学習・技術記事</x:v>
+      </x:c>
+      <x:c r="D69" s="11" t="str">
+        <x:v>フランス語圏</x:v>
+      </x:c>
+      <x:c r="E69" s="11" t="str">
+        <x:v>非営利で査読付きチュートリアルを継承。</x:v>
+      </x:c>
+      <x:c r="F69" s="11"/>
+      <x:c r="G69" s="11" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H69" s="11" t="str">
+        <x:v>原文記載なし</x:v>
+      </x:c>
+      <x:c r="I69" s="11" t="str">
         <x:v>人数の公開値を確認できず</x:v>
       </x:c>
-      <x:c r="J67" s="19"/>
-      <x:c r="K67" s="18" t="str">
+      <x:c r="J69" s="16"/>
+      <x:c r="K69" s="11" t="str">
         <x:v>未確認</x:v>
       </x:c>
-      <x:c r="L67" s="18" t="str">
+      <x:c r="L69" s="11" t="str">
         <x:v>未確認</x:v>
       </x:c>
-      <x:c r="M67" s="18" t="str"/>
-      <x:c r="N67" s="18" t="str">
+      <x:c r="M69" s="11"/>
+      <x:c r="N69" s="11" t="str">
         <x:v>基準時点を特定できず</x:v>
       </x:c>
-      <x:c r="O67" s="18" t="str">
+      <x:c r="O69" s="11" t="str">
         <x:v>公開値未確認</x:v>
       </x:c>
-      <x:c r="P67" s="18" t="str">
-        <x:v>https://eleduck.com/</x:v>
-      </x:c>
-      <x:c r="Q67" s="18" t="str">
-        <x:v>人数なし／初期1,000人獲得は用途例</x:v>
-      </x:c>
-      <x:c r="R67" s="18" t="str">
-        <x:v>公式の案内・規約・群組を調査したが総会員数の公開値は確認できず。Geminiの初期1,000人獲得は利用例の目標でサイト規模ではない。</x:v>
-      </x:c>
-      <x:c r="S67" s="20" t="d">
+      <x:c r="P69" s="11" t="str">
+        <x:v>https://zestedesavoir.com/</x:v>
+      </x:c>
+      <x:c r="Q69" s="11" t="str">
+        <x:v>定量的な人数記載なし</x:v>
+      </x:c>
+      <x:c r="R69" s="11" t="str">
+        <x:v>公式サイトはロボット制限により本文を取得できず。登録者数・MAUとも一次確認できず。</x:v>
+      </x:c>
+      <x:c r="S69" s="17" t="d">
         <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="68" ht="60" customHeight="1">
-      <x:c r="A68" s="11" t="str">
-        <x:v>P63</x:v>
-      </x:c>
-      <x:c r="B68" s="11" t="str">
-        <x:v>CSDN</x:v>
-      </x:c>
-      <x:c r="C68" s="11" t="str">
-        <x:v>技術記事・ブログ</x:v>
-      </x:c>
-      <x:c r="D68" s="11" t="str">
-        <x:v>中国</x:v>
-      </x:c>
-      <x:c r="E68" s="11" t="str">
-        <x:v>中国語技術ブログと備忘録の蓄積。</x:v>
-      </x:c>
-      <x:c r="F68" s="11" t="str"/>
-      <x:c r="G68" s="11" t="str">
+    <x:row r="70" ht="60" customHeight="1">
+      <x:c r="A70" s="12" t="str">
+        <x:v>P66</x:v>
+      </x:c>
+      <x:c r="B70" s="12" t="str">
+        <x:v>OpenClassrooms</x:v>
+      </x:c>
+      <x:c r="C70" s="12" t="str">
+        <x:v>教育・採用</x:v>
+      </x:c>
+      <x:c r="D70" s="12" t="str">
+        <x:v>フランス発・国際</x:v>
+      </x:c>
+      <x:c r="E70" s="12" t="str">
+        <x:v>旧チュートリアル共有サイトから商業教育へ転換。</x:v>
+      </x:c>
+      <x:c r="F70" s="12" t="str">
+        <x:v>旧Site du Zéro</x:v>
+      </x:c>
+      <x:c r="G70" s="12" t="str">
         <x:v>R2</x:v>
       </x:c>
-      <x:c r="H68" s="11" t="str">
+      <x:c r="H70" s="12" t="str">
         <x:v>原文記載なし</x:v>
       </x:c>
-      <x:c r="I68" s="11" t="str">
-        <x:v>登録会員</x:v>
-      </x:c>
-      <x:c r="J68" s="16" t="n">
-        <x:v>48000000</x:v>
-      </x:c>
-      <x:c r="K68" s="11" t="str">
+      <x:c r="I70" s="12" t="str">
+        <x:v>年間のキャリア成果報告者</x:v>
+      </x:c>
+      <x:c r="J70" s="23" t="n">
+        <x:v>43242</x:v>
+      </x:c>
+      <x:c r="K70" s="12" t="str">
+        <x:v>人/年（利用規模の補助指標）</x:v>
+      </x:c>
+      <x:c r="L70" s="12" t="str">
+        <x:v>全登録者・MAUは未確認</x:v>
+      </x:c>
+      <x:c r="M70" s="12"/>
+      <x:c r="N70" s="12" t="str">
+        <x:v>2025年実績・2026 Mission Report</x:v>
+      </x:c>
+      <x:c r="O70" s="12" t="str">
+        <x:v>公式報告・補助指標</x:v>
+      </x:c>
+      <x:c r="P70" s="12" t="str">
+        <x:v>https://blog.en.openclassrooms.com/post/impact-as-a-strategic-lever-not-just-a-showcase-openclassrooms-publishes-its-2026-mission-report</x:v>
+      </x:c>
+      <x:c r="Q70" s="12" t="str">
+        <x:v>定量的な人数記載なし</x:v>
+      </x:c>
+      <x:c r="R70" s="12" t="str">
+        <x:v>就職・昇進・起業等の成果自己申告者で、全利用者数ではない。2020年の月間訪問者など古い数値を現在のMAUとして混用しない。</x:v>
+      </x:c>
+      <x:c r="S70" s="24" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="71" ht="60" customHeight="1">
+      <x:c r="A71" s="11" t="str">
+        <x:v>P67</x:v>
+      </x:c>
+      <x:c r="B71" s="11" t="str">
+        <x:v>Les Pépites Tech</x:v>
+      </x:c>
+      <x:c r="C71" s="11" t="str">
+        <x:v>製品・スタートアップ公開</x:v>
+      </x:c>
+      <x:c r="D71" s="11" t="str">
+        <x:v>フランス・フランス語圏</x:v>
+      </x:c>
+      <x:c r="E71" s="11" t="str">
+        <x:v>French Techと結び付いた製品ディレクトリ。</x:v>
+      </x:c>
+      <x:c r="F71" s="11" t="str">
+        <x:v>lespepitestech.com</x:v>
+      </x:c>
+      <x:c r="G71" s="11" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H71" s="11" t="str">
+        <x:v>https://lespepitestech.com/</x:v>
+      </x:c>
+      <x:c r="I71" s="11" t="str">
+        <x:v>ディレクトリ掲載スタートアップ</x:v>
+      </x:c>
+      <x:c r="J71" s="16" t="n">
+        <x:v>4237</x:v>
+      </x:c>
+      <x:c r="K71" s="11" t="str">
+        <x:v>社（Grand Parisページ表示）</x:v>
+      </x:c>
+      <x:c r="L71" s="11" t="str">
+        <x:v>登録者・MAUは未確認</x:v>
+      </x:c>
+      <x:c r="M71" s="11"/>
+      <x:c r="N71" s="11" t="str">
+        <x:v>掲載時点不明・2026-10-21確認</x:v>
+      </x:c>
+      <x:c r="O71" s="11" t="str">
+        <x:v>公式確認・対象範囲注意</x:v>
+      </x:c>
+      <x:c r="P71" s="11" t="str">
+        <x:v>https://lespepitestech.com/french-tech-hub/french-tech-grand-paris</x:v>
+      </x:c>
+      <x:c r="Q71" s="11" t="str">
+        <x:v>掲載4,237社以上・13首都・38拠点</x:v>
+      </x:c>
+      <x:c r="R71" s="11" t="str">
+        <x:v>4237はGrand Parisページ上の表示値。全地域合計か地域限定かは確認できず、個人ユーザー数でもない。Geminiの全体規模という説明とは区別。</x:v>
+      </x:c>
+      <x:c r="S71" s="17" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="72" ht="60" customHeight="1">
+      <x:c r="A72" s="12" t="str">
+        <x:v>P68</x:v>
+      </x:c>
+      <x:c r="B72" s="12" t="str">
+        <x:v>WeLoveDevs.com</x:v>
+      </x:c>
+      <x:c r="C72" s="12" t="str">
+        <x:v>キャリア・技術記事</x:v>
+      </x:c>
+      <x:c r="D72" s="12" t="str">
+        <x:v>フランス</x:v>
+      </x:c>
+      <x:c r="E72" s="12" t="str">
+        <x:v>技術評価とポートフォリオを採用につなぐ。</x:v>
+      </x:c>
+      <x:c r="F72" s="12" t="str">
+        <x:v>WeLoveDevs</x:v>
+      </x:c>
+      <x:c r="G72" s="12" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H72" s="12" t="str">
+        <x:v>https://welovedevs.com/</x:v>
+      </x:c>
+      <x:c r="I72" s="12" t="str">
+        <x:v>利用・信頼する企業</x:v>
+      </x:c>
+      <x:c r="J72" s="23" t="n">
+        <x:v>3000</x:v>
+      </x:c>
+      <x:c r="K72" s="12" t="str">
+        <x:v>社</x:v>
+      </x:c>
+      <x:c r="L72" s="12" t="str">
+        <x:v>月間訪問者4万人超はGemini参考であり、今回公式一次確認できず。</x:v>
+      </x:c>
+      <x:c r="M72" s="12"/>
+      <x:c r="N72" s="12" t="str">
+        <x:v>掲載時点不明・2026-10-21確認</x:v>
+      </x:c>
+      <x:c r="O72" s="12" t="str">
+        <x:v>公式サービスサイトの自己申告</x:v>
+      </x:c>
+      <x:c r="P72" s="12" t="str">
+        <x:v>https://coderstests.com/fr/</x:v>
+      </x:c>
+      <x:c r="Q72" s="12" t="str">
+        <x:v>月間訪問4万人以上・企業2,500〜3,000社</x:v>
+      </x:c>
+      <x:c r="R72" s="12" t="str">
+        <x:v>CodersTests公式フッターがWeLoveDevsをtrusted by 3000 companiesと説明。開発者3万人はCodersTestsのネットワーク指標に分離。</x:v>
+      </x:c>
+      <x:c r="S72" s="24" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="73" ht="60" customHeight="1">
+      <x:c r="A73" s="11" t="str">
+        <x:v>P69</x:v>
+      </x:c>
+      <x:c r="B73" s="11" t="str">
+        <x:v>CodersTests</x:v>
+      </x:c>
+      <x:c r="C73" s="11" t="str">
+        <x:v>技術評価・キャリア</x:v>
+      </x:c>
+      <x:c r="D73" s="11" t="str">
+        <x:v>フランス</x:v>
+      </x:c>
+      <x:c r="E73" s="11" t="str">
+        <x:v>専門家の技術テストと実績証明。</x:v>
+      </x:c>
+      <x:c r="F73" s="11"/>
+      <x:c r="G73" s="11" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H73" s="11" t="str">
+        <x:v>原文記載なし</x:v>
+      </x:c>
+      <x:c r="I73" s="11" t="str">
+        <x:v>開発者ネットワーク</x:v>
+      </x:c>
+      <x:c r="J73" s="16" t="n">
+        <x:v>30000</x:v>
+      </x:c>
+      <x:c r="K73" s="11" t="str">
         <x:v>超・人</x:v>
       </x:c>
-      <x:c r="L68" s="11" t="str">
+      <x:c r="L73" s="11" t="str">
         <x:v>MAU/DAUは未確認</x:v>
       </x:c>
-      <x:c r="M68" s="11" t="str">
-        <x:v>年平均新規利用者700万人、企業顧客・パートナー1,000社以上</x:v>
-      </x:c>
-      <x:c r="N68" s="11" t="str">
+      <x:c r="M73" s="11" t="str">
+        <x:v>評価問題プール3,000問以上</x:v>
+      </x:c>
+      <x:c r="N73" s="11" t="str">
         <x:v>掲載時点不明・2026-10-21確認</x:v>
       </x:c>
-      <x:c r="O68" s="11" t="str">
-        <x:v>公式確認</x:v>
-      </x:c>
-      <x:c r="P68" s="11" t="str">
-        <x:v>https://www.csdn.net/company/index.html</x:v>
-      </x:c>
-      <x:c r="Q68" s="11" t="str">
+      <x:c r="O73" s="11" t="str">
+        <x:v>公式確認・定義注意</x:v>
+      </x:c>
+      <x:c r="P73" s="11" t="str">
+        <x:v>https://coderstests.com/fr/</x:v>
+      </x:c>
+      <x:c r="Q73" s="11" t="str">
+        <x:v>開発者3万人以上・技術テスト100種以上</x:v>
+      </x:c>
+      <x:c r="R73" s="11" t="str">
+        <x:v>公式はnetwork of 30,000+ developers。登録受験者数と断定しない。</x:v>
+      </x:c>
+      <x:c r="S73" s="17" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="74" ht="60" customHeight="1">
+      <x:c r="A74" s="12" t="str">
+        <x:v>P70</x:v>
+      </x:c>
+      <x:c r="B74" s="12" t="str">
+        <x:v>Velog</x:v>
+      </x:c>
+      <x:c r="C74" s="12" t="str">
+        <x:v>技術ブログ</x:v>
+      </x:c>
+      <x:c r="D74" s="12" t="str">
+        <x:v>韓国語圏</x:v>
+      </x:c>
+      <x:c r="E74" s="12" t="str">
+        <x:v>韓国語とMarkdownの執筆体験に特化。</x:v>
+      </x:c>
+      <x:c r="F74" s="12" t="str">
+        <x:v>velog.io</x:v>
+      </x:c>
+      <x:c r="G74" s="12" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H74" s="12" t="str">
+        <x:v>https://velog.io/</x:v>
+      </x:c>
+      <x:c r="I74" s="12" t="str">
+        <x:v>人数の公開値を確認できず</x:v>
+      </x:c>
+      <x:c r="J74" s="23"/>
+      <x:c r="K74" s="12" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="L74" s="12" t="str">
+        <x:v>未確認</x:v>
+      </x:c>
+      <x:c r="M74" s="12"/>
+      <x:c r="N74" s="12" t="str">
+        <x:v>基準時点を特定できず</x:v>
+      </x:c>
+      <x:c r="O74" s="12" t="str">
+        <x:v>公開値未確認</x:v>
+      </x:c>
+      <x:c r="P74" s="12" t="str">
+        <x:v>https://velog.io/</x:v>
+      </x:c>
+      <x:c r="Q74" s="12" t="str">
         <x:v>定量的な人数記載なし</x:v>
       </x:c>
-      <x:c r="R68" s="11" t="str">
-        <x:v>公式会社案内の4,800万人超。ユーザー投稿にある5,100万人等を公式値と混同しない。</x:v>
-      </x:c>
-      <x:c r="S68" s="17" t="d">
+      <x:c r="R74" s="12" t="str">
+        <x:v>公式・開発者情報を検索したがサイト全体の登録者・MAU値は確認できず。利用者の記事内の別アプリやVelog Stats拡張のユーザー数は転記しない。</x:v>
+      </x:c>
+      <x:c r="S74" s="24" t="d">
         <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
-    <x:row r="69" ht="60" customHeight="1">
-      <x:c r="A69" s="12" t="str">
-        <x:v>P64</x:v>
-      </x:c>
-      <x:c r="B69" s="12" t="str">
-        <x:v>Developpez.com</x:v>
-      </x:c>
-      <x:c r="C69" s="12" t="str">
-        <x:v>技術記事・Q&amp;A・学習</x:v>
-      </x:c>
-      <x:c r="D69" s="12" t="str">
-        <x:v>フランス語圏</x:v>
-      </x:c>
-      <x:c r="E69" s="12" t="str">
-        <x:v>ボランティアが運営する老舗の技術情報共有。</x:v>
-      </x:c>
-      <x:c r="F69" s="12" t="str">
-        <x:v>Le Club des Développeurs et IT Pro</x:v>
-      </x:c>
-      <x:c r="G69" s="12" t="str">
+    <x:row r="75" ht="60" customHeight="1">
+      <x:c r="A75" s="11" t="str">
+        <x:v>P71</x:v>
+      </x:c>
+      <x:c r="B75" s="11" t="str">
+        <x:v>Disquiet</x:v>
+      </x:c>
+      <x:c r="C75" s="11" t="str">
+        <x:v>製品公開・開発者SNS</x:v>
+      </x:c>
+      <x:c r="D75" s="11" t="str">
+        <x:v>韓国</x:v>
+      </x:c>
+      <x:c r="E75" s="11" t="str">
+        <x:v>製品と日々の開発記録を連動させる。</x:v>
+      </x:c>
+      <x:c r="F75" s="11" t="str">
+        <x:v>disquiet.io / 디스콰이엇 / メイカーログ / Makerlog</x:v>
+      </x:c>
+      <x:c r="G75" s="11" t="str">
         <x:v>R2</x:v>
       </x:c>
-      <x:c r="H69" s="12" t="str">
-        <x:v>https://developpez.com/</x:v>
-      </x:c>
-      <x:c r="I69" s="18" t="str">
-        <x:v>会員数（歴史値）</x:v>
-      </x:c>
-      <x:c r="J69" s="19" t="n">
-        <x:v>750000</x:v>
-      </x:c>
-      <x:c r="K69" s="18" t="str">
-        <x:v>人</x:v>
-      </x:c>
-      <x:c r="L69" s="18" t="str">
-        <x:v>月間最大400万UV・1,200万PV（歴史値）</x:v>
-      </x:c>
-      <x:c r="M69" s="18" t="str">
-        <x:v>2,000フォーラム、最大5,000投稿/日（同じ公表）</x:v>
-      </x:c>
-      <x:c r="N69" s="18" t="str">
-        <x:v>2017年公表記事・現在値は未確認</x:v>
-      </x:c>
-      <x:c r="O69" s="18" t="str">
-        <x:v>公式運営投稿・歴史値</x:v>
-      </x:c>
-      <x:c r="P69" s="18" t="str">
-        <x:v>https://www.developpez.net/forums/i1675688/club-professionnels-informatique/actualites/croissance-annuelle-16-reseau-social-club-developpez-com/</x:v>
-      </x:c>
-      <x:c r="Q69" s="18" t="str">
-        <x:v>月間最大400万UU・5,000投稿/日・14,000記事</x:v>
-      </x:c>
-      <x:c r="R69" s="18" t="str">
-        <x:v>原レポートの月間400万UUには古い公表と一致する値が含まれる。2026年の実測値とは扱わない。</x:v>
-      </x:c>
-      <x:c r="S69" s="20" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="70" ht="60" customHeight="1">
-      <x:c r="A70" s="11" t="str">
-        <x:v>P65</x:v>
-      </x:c>
-      <x:c r="B70" s="11" t="str">
-        <x:v>Zeste de Savoir</x:v>
-      </x:c>
-      <x:c r="C70" s="11" t="str">
-        <x:v>学習・技術記事</x:v>
-      </x:c>
-      <x:c r="D70" s="11" t="str">
-        <x:v>フランス語圏</x:v>
-      </x:c>
-      <x:c r="E70" s="11" t="str">
-        <x:v>非営利で査読付きチュートリアルを継承。</x:v>
-      </x:c>
-      <x:c r="F70" s="11" t="str"/>
-      <x:c r="G70" s="11" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H70" s="11" t="str">
-        <x:v>原文記載なし</x:v>
-      </x:c>
-      <x:c r="I70" s="11" t="str">
-        <x:v>人数の公開値を確認できず</x:v>
-      </x:c>
-      <x:c r="J70" s="16"/>
-      <x:c r="K70" s="11" t="str">
-        <x:v>未確認</x:v>
-      </x:c>
-      <x:c r="L70" s="11" t="str">
-        <x:v>未確認</x:v>
-      </x:c>
-      <x:c r="M70" s="11" t="str"/>
-      <x:c r="N70" s="11" t="str">
-        <x:v>基準時点を特定できず</x:v>
-      </x:c>
-      <x:c r="O70" s="11" t="str">
-        <x:v>公開値未確認</x:v>
-      </x:c>
-      <x:c r="P70" s="11" t="str">
-        <x:v>https://zestedesavoir.com/</x:v>
-      </x:c>
-      <x:c r="Q70" s="11" t="str">
-        <x:v>定量的な人数記載なし</x:v>
-      </x:c>
-      <x:c r="R70" s="11" t="str">
-        <x:v>公式サイトはロボット制限により本文を取得できず。登録者数・MAUとも一次確認できず。</x:v>
-      </x:c>
-      <x:c r="S70" s="17" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="71" ht="60" customHeight="1">
-      <x:c r="A71" s="12" t="str">
-        <x:v>P66</x:v>
-      </x:c>
-      <x:c r="B71" s="12" t="str">
-        <x:v>OpenClassrooms</x:v>
-      </x:c>
-      <x:c r="C71" s="12" t="str">
-        <x:v>教育・採用</x:v>
-      </x:c>
-      <x:c r="D71" s="12" t="str">
-        <x:v>フランス発・国際</x:v>
-      </x:c>
-      <x:c r="E71" s="12" t="str">
-        <x:v>旧チュートリアル共有サイトから商業教育へ転換。</x:v>
-      </x:c>
-      <x:c r="F71" s="12" t="str">
-        <x:v>旧Site du Zéro</x:v>
-      </x:c>
-      <x:c r="G71" s="12" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H71" s="12" t="str">
-        <x:v>原文記載なし</x:v>
-      </x:c>
-      <x:c r="I71" s="18" t="str">
-        <x:v>年間のキャリア成果報告者</x:v>
-      </x:c>
-      <x:c r="J71" s="19" t="n">
-        <x:v>43242</x:v>
-      </x:c>
-      <x:c r="K71" s="18" t="str">
-        <x:v>人/年（利用規模の補助指標）</x:v>
-      </x:c>
-      <x:c r="L71" s="18" t="str">
-        <x:v>全登録者・MAUは未確認</x:v>
-      </x:c>
-      <x:c r="M71" s="18" t="str"/>
-      <x:c r="N71" s="18" t="str">
-        <x:v>2025年実績・2026 Mission Report</x:v>
-      </x:c>
-      <x:c r="O71" s="18" t="str">
-        <x:v>公式報告・補助指標</x:v>
-      </x:c>
-      <x:c r="P71" s="18" t="str">
-        <x:v>https://blog.en.openclassrooms.com/post/impact-as-a-strategic-lever-not-just-a-showcase-openclassrooms-publishes-its-2026-mission-report</x:v>
-      </x:c>
-      <x:c r="Q71" s="18" t="str">
-        <x:v>定量的な人数記載なし</x:v>
-      </x:c>
-      <x:c r="R71" s="18" t="str">
-        <x:v>就職・昇進・起業等の成果自己申告者で、全利用者数ではない。2020年の月間訪問者など古い数値を現在のMAUとして混用しない。</x:v>
-      </x:c>
-      <x:c r="S71" s="20" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="72" ht="60" customHeight="1">
-      <x:c r="A72" s="11" t="str">
-        <x:v>P67</x:v>
-      </x:c>
-      <x:c r="B72" s="11" t="str">
-        <x:v>Les Pépites Tech</x:v>
-      </x:c>
-      <x:c r="C72" s="11" t="str">
-        <x:v>製品・スタートアップ公開</x:v>
-      </x:c>
-      <x:c r="D72" s="11" t="str">
-        <x:v>フランス・フランス語圏</x:v>
-      </x:c>
-      <x:c r="E72" s="11" t="str">
-        <x:v>French Techと結び付いた製品ディレクトリ。</x:v>
-      </x:c>
-      <x:c r="F72" s="11" t="str">
-        <x:v>lespepitestech.com</x:v>
-      </x:c>
-      <x:c r="G72" s="11" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H72" s="11" t="str">
-        <x:v>https://lespepitestech.com/</x:v>
-      </x:c>
-      <x:c r="I72" s="11" t="str">
-        <x:v>ディレクトリ掲載スタートアップ</x:v>
-      </x:c>
-      <x:c r="J72" s="16" t="n">
-        <x:v>4237</x:v>
-      </x:c>
-      <x:c r="K72" s="11" t="str">
-        <x:v>社（Grand Parisページ表示）</x:v>
-      </x:c>
-      <x:c r="L72" s="11" t="str">
-        <x:v>登録者・MAUは未確認</x:v>
-      </x:c>
-      <x:c r="M72" s="11" t="str"/>
-      <x:c r="N72" s="11" t="str">
-        <x:v>掲載時点不明・2026-10-21確認</x:v>
-      </x:c>
-      <x:c r="O72" s="11" t="str">
-        <x:v>公式確認・対象範囲注意</x:v>
-      </x:c>
-      <x:c r="P72" s="11" t="str">
-        <x:v>https://lespepitestech.com/french-tech-hub/french-tech-grand-paris</x:v>
-      </x:c>
-      <x:c r="Q72" s="11" t="str">
-        <x:v>掲載4,237社以上・13首都・38拠点</x:v>
-      </x:c>
-      <x:c r="R72" s="11" t="str">
-        <x:v>4237はGrand Parisページ上の表示値。全地域合計か地域限定かは確認できず、個人ユーザー数でもない。Geminiの全体規模という説明とは区別。</x:v>
-      </x:c>
-      <x:c r="S72" s="17" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="73" ht="60" customHeight="1">
-      <x:c r="A73" s="12" t="str">
-        <x:v>P68</x:v>
-      </x:c>
-      <x:c r="B73" s="12" t="str">
-        <x:v>WeLoveDevs.com</x:v>
-      </x:c>
-      <x:c r="C73" s="12" t="str">
-        <x:v>キャリア・技術記事</x:v>
-      </x:c>
-      <x:c r="D73" s="12" t="str">
-        <x:v>フランス</x:v>
-      </x:c>
-      <x:c r="E73" s="12" t="str">
-        <x:v>技術評価とポートフォリオを採用につなぐ。</x:v>
-      </x:c>
-      <x:c r="F73" s="12" t="str">
-        <x:v>WeLoveDevs</x:v>
-      </x:c>
-      <x:c r="G73" s="12" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H73" s="12" t="str">
-        <x:v>https://welovedevs.com/</x:v>
-      </x:c>
-      <x:c r="I73" s="18" t="str">
-        <x:v>利用・信頼する企業</x:v>
-      </x:c>
-      <x:c r="J73" s="19" t="n">
-        <x:v>3000</x:v>
-      </x:c>
-      <x:c r="K73" s="18" t="str">
-        <x:v>社</x:v>
-      </x:c>
-      <x:c r="L73" s="18" t="str">
-        <x:v>月間訪問者4万人超はGemini参考であり、今回公式一次確認できず。</x:v>
-      </x:c>
-      <x:c r="M73" s="18" t="str"/>
-      <x:c r="N73" s="18" t="str">
-        <x:v>掲載時点不明・2026-10-21確認</x:v>
-      </x:c>
-      <x:c r="O73" s="18" t="str">
-        <x:v>公式サービスサイトの自己申告</x:v>
-      </x:c>
-      <x:c r="P73" s="18" t="str">
-        <x:v>https://coderstests.com/fr/</x:v>
-      </x:c>
-      <x:c r="Q73" s="18" t="str">
-        <x:v>月間訪問4万人以上・企業2,500〜3,000社</x:v>
-      </x:c>
-      <x:c r="R73" s="18" t="str">
-        <x:v>CodersTests公式フッターがWeLoveDevsをtrusted by 3000 companiesと説明。開発者3万人はCodersTestsのネットワーク指標に分離。</x:v>
-      </x:c>
-      <x:c r="S73" s="20" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="74" ht="60" customHeight="1">
-      <x:c r="A74" s="11" t="str">
-        <x:v>P69</x:v>
-      </x:c>
-      <x:c r="B74" s="11" t="str">
-        <x:v>CodersTests</x:v>
-      </x:c>
-      <x:c r="C74" s="11" t="str">
-        <x:v>技術評価・キャリア</x:v>
-      </x:c>
-      <x:c r="D74" s="11" t="str">
-        <x:v>フランス</x:v>
-      </x:c>
-      <x:c r="E74" s="11" t="str">
-        <x:v>専門家の技術テストと実績証明。</x:v>
-      </x:c>
-      <x:c r="F74" s="11" t="str"/>
-      <x:c r="G74" s="11" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H74" s="11" t="str">
-        <x:v>原文記載なし</x:v>
-      </x:c>
-      <x:c r="I74" s="11" t="str">
-        <x:v>開発者ネットワーク</x:v>
-      </x:c>
-      <x:c r="J74" s="16" t="n">
-        <x:v>30000</x:v>
-      </x:c>
-      <x:c r="K74" s="11" t="str">
-        <x:v>超・人</x:v>
-      </x:c>
-      <x:c r="L74" s="11" t="str">
-        <x:v>MAU/DAUは未確認</x:v>
-      </x:c>
-      <x:c r="M74" s="11" t="str">
-        <x:v>評価問題プール3,000問以上</x:v>
-      </x:c>
-      <x:c r="N74" s="11" t="str">
-        <x:v>掲載時点不明・2026-10-21確認</x:v>
-      </x:c>
-      <x:c r="O74" s="11" t="str">
-        <x:v>公式確認・定義注意</x:v>
-      </x:c>
-      <x:c r="P74" s="11" t="str">
-        <x:v>https://coderstests.com/fr/</x:v>
-      </x:c>
-      <x:c r="Q74" s="11" t="str">
-        <x:v>開発者3万人以上・技術テスト100種以上</x:v>
-      </x:c>
-      <x:c r="R74" s="11" t="str">
-        <x:v>公式はnetwork of 30,000+ developers。登録受験者数と断定しない。</x:v>
-      </x:c>
-      <x:c r="S74" s="17" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="75" ht="60" customHeight="1">
-      <x:c r="A75" s="12" t="str">
-        <x:v>P70</x:v>
-      </x:c>
-      <x:c r="B75" s="12" t="str">
-        <x:v>Velog</x:v>
-      </x:c>
-      <x:c r="C75" s="12" t="str">
-        <x:v>技術ブログ</x:v>
-      </x:c>
-      <x:c r="D75" s="12" t="str">
-        <x:v>韓国語圏</x:v>
-      </x:c>
-      <x:c r="E75" s="12" t="str">
-        <x:v>韓国語とMarkdownの執筆体験に特化。</x:v>
-      </x:c>
-      <x:c r="F75" s="12" t="str">
-        <x:v>velog.io</x:v>
-      </x:c>
-      <x:c r="G75" s="12" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H75" s="12" t="str">
-        <x:v>https://velog.io/</x:v>
-      </x:c>
-      <x:c r="I75" s="18" t="str">
-        <x:v>人数の公開値を確認できず</x:v>
-      </x:c>
-      <x:c r="J75" s="19"/>
-      <x:c r="K75" s="18" t="str">
-        <x:v>未確認</x:v>
-      </x:c>
-      <x:c r="L75" s="18" t="str">
-        <x:v>未確認</x:v>
-      </x:c>
-      <x:c r="M75" s="18" t="str"/>
-      <x:c r="N75" s="18" t="str">
-        <x:v>基準時点を特定できず</x:v>
-      </x:c>
-      <x:c r="O75" s="18" t="str">
-        <x:v>公開値未確認</x:v>
-      </x:c>
-      <x:c r="P75" s="18" t="str">
-        <x:v>https://velog.io/</x:v>
-      </x:c>
-      <x:c r="Q75" s="18" t="str">
-        <x:v>定量的な人数記載なし</x:v>
-      </x:c>
-      <x:c r="R75" s="18" t="str">
-        <x:v>公式・開発者情報を検索したがサイト全体の登録者・MAU値は確認できず。利用者の記事内の別アプリやVelog Stats拡張のユーザー数は転記しない。</x:v>
-      </x:c>
-      <x:c r="S75" s="20" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="76" ht="60" customHeight="1">
-      <x:c r="A76" s="11" t="str">
-        <x:v>P71</x:v>
-      </x:c>
-      <x:c r="B76" s="11" t="str">
-        <x:v>Disquiet</x:v>
-      </x:c>
-      <x:c r="C76" s="11" t="str">
-        <x:v>製品公開・開発者SNS</x:v>
-      </x:c>
-      <x:c r="D76" s="11" t="str">
-        <x:v>韓国</x:v>
-      </x:c>
-      <x:c r="E76" s="11" t="str">
-        <x:v>製品と日々の開発記録を連動させる。</x:v>
-      </x:c>
-      <x:c r="F76" s="11" t="str">
-        <x:v>disquiet.io / 디스콰이엇 / メイカーログ / Makerlog</x:v>
-      </x:c>
-      <x:c r="G76" s="11" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H76" s="11" t="str">
+      <x:c r="H75" s="11" t="str">
         <x:v>https://disquiet.io/</x:v>
       </x:c>
-      <x:c r="I76" s="11" t="str">
+      <x:c r="I75" s="11" t="str">
         <x:v>月間新規製品登録（Gemini参考）</x:v>
       </x:c>
-      <x:c r="J76" s="16" t="n">
+      <x:c r="J75" s="16" t="n">
         <x:v>200</x:v>
       </x:c>
-      <x:c r="K76" s="11" t="str">
+      <x:c r="K75" s="11" t="str">
         <x:v>以上・件/月</x:v>
       </x:c>
-      <x:c r="L76" s="11" t="str">
+      <x:c r="L75" s="11" t="str">
         <x:v>会員数・MAUは未確認</x:v>
       </x:c>
-      <x:c r="M76" s="11" t="str"/>
-      <x:c r="N76" s="11" t="str">
+      <x:c r="M75" s="11"/>
+      <x:c r="N75" s="11" t="str">
         <x:v>2023年基準（Geminiの記載）</x:v>
       </x:c>
-      <x:c r="O76" s="11" t="str">
+      <x:c r="O75" s="11" t="str">
         <x:v>レポート参考・一次未確認</x:v>
       </x:c>
-      <x:c r="P76" s="11" t="str">
+      <x:c r="P75" s="11" t="str">
         <x:v>https://gemini.google.com/share/9089e9cfab60?social_preview=false&amp;skid=5696a754-a556-4584-af0e-e53a5b1205ee
 https://blog.disquiet.io/post/disquiet-mission-and-vision</x:v>
       </x:c>
-      <x:c r="Q76" s="11" t="str">
+      <x:c r="Q75" s="11" t="str">
         <x:v>月間新規製品200件以上（2023年基準）</x:v>
       </x:c>
-      <x:c r="R76" s="11" t="str">
+      <x:c r="R75" s="11" t="str">
         <x:v>月間200件は製品投稿数であり利用者人数ではない。公式創業者記事の検索から最新の全体人数は確認できず。</x:v>
       </x:c>
-      <x:c r="S76" s="17" t="d">
+      <x:c r="S75" s="17" t="d">
         <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
+    <x:row r="76" ht="60" customHeight="1">
+      <x:c r="A76" s="12" t="str">
+        <x:v>P72</x:v>
+      </x:c>
+      <x:c r="B76" s="12" t="str">
+        <x:v>OKKY</x:v>
+      </x:c>
+      <x:c r="C76" s="12" t="str">
+        <x:v>Q&amp;A・キャリア</x:v>
+      </x:c>
+      <x:c r="D76" s="12" t="str">
+        <x:v>韓国</x:v>
+      </x:c>
+      <x:c r="E76" s="12" t="str">
+        <x:v>韓国エンジニアの質問解決と実務経験共有。</x:v>
+      </x:c>
+      <x:c r="F76" s="12" t="str">
+        <x:v>okky.kr</x:v>
+      </x:c>
+      <x:c r="G76" s="12" t="str">
+        <x:v>R2</x:v>
+      </x:c>
+      <x:c r="H76" s="12" t="str">
+        <x:v>https://okky.kr/</x:v>
+      </x:c>
+      <x:c r="I76" s="12" t="str">
+        <x:v>登録会員</x:v>
+      </x:c>
+      <x:c r="J76" s="23" t="n">
+        <x:v>180000</x:v>
+      </x:c>
+      <x:c r="K76" s="12" t="str">
+        <x:v>超・人</x:v>
+      </x:c>
+      <x:c r="L76" s="12" t="str">
+        <x:v>月間訪問者70万人、月間700万PV（会社案内の表示値）</x:v>
+      </x:c>
+      <x:c r="M76" s="12" t="str">
+        <x:v>知識・ライフ関連コンテンツ1,000万件</x:v>
+      </x:c>
+      <x:c r="N76" s="12" t="str">
+        <x:v>会員18万人：2025年沿革／訪問者等：時点不明</x:v>
+      </x:c>
+      <x:c r="O76" s="12" t="str">
+        <x:v>公式確認</x:v>
+      </x:c>
+      <x:c r="P76" s="12" t="str">
+        <x:v>https://okky.kr/corp/about</x:v>
+      </x:c>
+      <x:c r="Q76" s="12" t="str">
+        <x:v>定量的な人数記載なし</x:v>
+      </x:c>
+      <x:c r="R76" s="12" t="str">
+        <x:v>沿革の2025年18万人超と、時点が明示されない訪問者・PVを分けて記録。</x:v>
+      </x:c>
+      <x:c r="S76" s="24" t="d">
+        <x:v>2026-10-21T00:00:00.000Z</x:v>
+      </x:c>
+    </x:row>
     <x:row r="77" ht="60" customHeight="1">
-      <x:c r="A77" s="12" t="str">
-        <x:v>P72</x:v>
-      </x:c>
-      <x:c r="B77" s="12" t="str">
-        <x:v>OKKY</x:v>
-      </x:c>
-      <x:c r="C77" s="12" t="str">
-        <x:v>Q&amp;A・キャリア</x:v>
-      </x:c>
-      <x:c r="D77" s="12" t="str">
-        <x:v>韓国</x:v>
-      </x:c>
-      <x:c r="E77" s="12" t="str">
-        <x:v>韓国エンジニアの質問解決と実務経験共有。</x:v>
-      </x:c>
-      <x:c r="F77" s="12" t="str">
-        <x:v>okky.kr</x:v>
-      </x:c>
-      <x:c r="G77" s="12" t="str">
+      <x:c r="A77" s="11" t="str">
+        <x:v>P73</x:v>
+      </x:c>
+      <x:c r="B77" s="11" t="str">
+        <x:v>Habr</x:v>
+      </x:c>
+      <x:c r="C77" s="11" t="str">
+        <x:v>技術記事・専門メディア</x:v>
+      </x:c>
+      <x:c r="D77" s="11" t="str">
+        <x:v>ロシア語圏</x:v>
+      </x:c>
+      <x:c r="E77" s="11" t="str">
+        <x:v>審査と評判、著者への金銭報酬を組み合わせる。</x:v>
+      </x:c>
+      <x:c r="F77" s="11" t="str">
+        <x:v>habr.com / 旧Habrahabr / ППА</x:v>
+      </x:c>
+      <x:c r="G77" s="11" t="str">
         <x:v>R2</x:v>
       </x:c>
-      <x:c r="H77" s="12" t="str">
-        <x:v>https://okky.kr/</x:v>
-      </x:c>
-      <x:c r="I77" s="18" t="str">
-        <x:v>登録会員</x:v>
-      </x:c>
-      <x:c r="J77" s="19" t="n">
-        <x:v>180000</x:v>
-      </x:c>
-      <x:c r="K77" s="18" t="str">
-        <x:v>超・人</x:v>
-      </x:c>
-      <x:c r="L77" s="18" t="str">
-        <x:v>月間訪問者70万人、月間700万PV（会社案内の表示値）</x:v>
-      </x:c>
-      <x:c r="M77" s="18" t="str">
-        <x:v>知識・ライフ関連コンテンツ1,000万件</x:v>
-      </x:c>
-      <x:c r="N77" s="18" t="str">
-        <x:v>会員18万人：2025年沿革／訪問者等：時点不明</x:v>
-      </x:c>
-      <x:c r="O77" s="18" t="str">
+      <x:c r="H77" s="11" t="str">
+        <x:v>https://habr.com/</x:v>
+      </x:c>
+      <x:c r="I77" s="11" t="str">
+        <x:v>月間利用者（公式表現）</x:v>
+      </x:c>
+      <x:c r="J77" s="16" t="n">
+        <x:v>13000000</x:v>
+      </x:c>
+      <x:c r="K77" s="11" t="str">
+        <x:v>超・人/月</x:v>
+      </x:c>
+      <x:c r="L77" s="11" t="str">
+        <x:v>公式会社案内で月間1,300万人超と記載</x:v>
+      </x:c>
+      <x:c r="M77" s="11"/>
+      <x:c r="N77" s="11" t="str">
+        <x:v>掲載時点不明・2026-10-21確認</x:v>
+      </x:c>
+      <x:c r="O77" s="11" t="str">
         <x:v>公式確認</x:v>
       </x:c>
-      <x:c r="P77" s="18" t="str">
-        <x:v>https://okky.kr/corp/about</x:v>
-      </x:c>
-      <x:c r="Q77" s="18" t="str">
+      <x:c r="P77" s="11" t="str">
+        <x:v>https://company.habr.com/en/</x:v>
+      </x:c>
+      <x:c r="Q77" s="11" t="str">
         <x:v>定量的な人数記載なし</x:v>
       </x:c>
-      <x:c r="R77" s="18" t="str">
-        <x:v>沿革の2025年18万人超と、時点が明示されない訪問者・PVを分けて記録。</x:v>
-      </x:c>
-      <x:c r="S77" s="20" t="d">
+      <x:c r="R77" s="11" t="str">
+        <x:v>旧スポンサー説明の月間800万UVとは別ページ・別時点。最新会社案内の13Mを採用し、登録会員数へ読み替えない。</x:v>
+      </x:c>
+      <x:c r="S77" s="17" t="d">
         <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="78" ht="60" customHeight="1">
-      <x:c r="A78" s="11" t="str">
-        <x:v>P73</x:v>
-      </x:c>
-      <x:c r="B78" s="11" t="str">
-        <x:v>Habr</x:v>
-      </x:c>
-      <x:c r="C78" s="11" t="str">
-        <x:v>技術記事・専門メディア</x:v>
-      </x:c>
-      <x:c r="D78" s="11" t="str">
-        <x:v>ロシア語圏</x:v>
-      </x:c>
-      <x:c r="E78" s="11" t="str">
-        <x:v>審査と評判、著者への金銭報酬を組み合わせる。</x:v>
-      </x:c>
-      <x:c r="F78" s="11" t="str">
-        <x:v>habr.com / 旧Habrahabr / ППА</x:v>
-      </x:c>
-      <x:c r="G78" s="11" t="str">
+      <x:c r="A78" s="12" t="str">
+        <x:v>P74</x:v>
+      </x:c>
+      <x:c r="B78" s="12" t="str">
+        <x:v>TabNews</x:v>
+      </x:c>
+      <x:c r="C78" s="12" t="str">
+        <x:v>技術記事・プロジェクト共有</x:v>
+      </x:c>
+      <x:c r="D78" s="12" t="str">
+        <x:v>ブラジル・ポルトガル語圏</x:v>
+      </x:c>
+      <x:c r="E78" s="12" t="str">
+        <x:v>OSSと二種類の貢献・広告指標でスパムを抑える。</x:v>
+      </x:c>
+      <x:c r="F78" s="12" t="str">
+        <x:v>tabnews.com.br / 原文比較表ではtabnews.br</x:v>
+      </x:c>
+      <x:c r="G78" s="12" t="str">
         <x:v>R2</x:v>
       </x:c>
-      <x:c r="H78" s="11" t="str">
-        <x:v>https://habr.com/</x:v>
-      </x:c>
-      <x:c r="I78" s="11" t="str">
-        <x:v>月間利用者（公式表現）</x:v>
-      </x:c>
-      <x:c r="J78" s="16" t="n">
-        <x:v>13000000</x:v>
-      </x:c>
-      <x:c r="K78" s="11" t="str">
-        <x:v>超・人/月</x:v>
-      </x:c>
-      <x:c r="L78" s="11" t="str">
-        <x:v>公式会社案内で月間1,300万人超と記載</x:v>
-      </x:c>
-      <x:c r="M78" s="11" t="str"/>
-      <x:c r="N78" s="11" t="str">
-        <x:v>掲載時点不明・2026-10-21確認</x:v>
-      </x:c>
-      <x:c r="O78" s="11" t="str">
-        <x:v>公式確認</x:v>
-      </x:c>
-      <x:c r="P78" s="11" t="str">
-        <x:v>https://company.habr.com/en/</x:v>
-      </x:c>
-      <x:c r="Q78" s="11" t="str">
-        <x:v>定量的な人数記載なし</x:v>
-      </x:c>
-      <x:c r="R78" s="11" t="str">
-        <x:v>旧スポンサー説明の月間800万UVとは別ページ・別時点。最新会社案内の13Mを採用し、登録会員数へ読み替えない。</x:v>
-      </x:c>
-      <x:c r="S78" s="17" t="d">
+      <x:c r="H78" s="12" t="str">
+        <x:v>https://tabnews.com.br/</x:v>
+      </x:c>
+      <x:c r="I78" s="12" t="str">
+        <x:v>有効化済み登録アカウント</x:v>
+      </x:c>
+      <x:c r="J78" s="23" t="n">
+        <x:v>45252</x:v>
+      </x:c>
+      <x:c r="K78" s="12" t="str">
+        <x:v>件・年末時点</x:v>
+      </x:c>
+      <x:c r="L78" s="12" t="str">
+        <x:v>2024年月平均ログイン2,595人・反応参加1,038人、日平均端末UV約5,700</x:v>
+      </x:c>
+      <x:c r="M78" s="12" t="str">
+        <x:v>2024年5,700,000PV。2,100,000訪問者は日次端末UVの年内合計。</x:v>
+      </x:c>
+      <x:c r="N78" s="12" t="str">
+        <x:v>登録数2024年末、活動・PV2024年実績</x:v>
+      </x:c>
+      <x:c r="O78" s="12" t="str">
+        <x:v>運営側の公開集計・歴史値</x:v>
+      </x:c>
+      <x:c r="P78" s="12" t="str">
+        <x:v>https://www.tabnews.com.br/FelipeBarso/tabnews-mais-de-2m-de-visitantes-e-5m-de-visualizacoes-em-2024</x:v>
+      </x:c>
+      <x:c r="Q78" s="12" t="str">
+        <x:v>人数なし／100 TabCashは通貨制度</x:v>
+      </x:c>
+      <x:c r="R78" s="12" t="str">
+        <x:v>有効化済み登録（cadastro ativo）はアクティブ利用の意味ではない。年間訪問者合計は年次の異なる人の数ではないと原文が明記。</x:v>
+      </x:c>
+      <x:c r="S78" s="24" t="d">
         <x:v>2026-10-21T00:00:00.000Z</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="60" customHeight="1">
-      <x:c r="A79" s="12" t="str">
-        <x:v>P74</x:v>
-      </x:c>
-      <x:c r="B79" s="12" t="str">
-        <x:v>TabNews</x:v>
-      </x:c>
-      <x:c r="C79" s="12" t="str">
-        <x:v>技術記事・プロジェクト共有</x:v>
-      </x:c>
-      <x:c r="D79" s="12" t="str">
-        <x:v>ブラジル・ポルトガル語圏</x:v>
-      </x:c>
-      <x:c r="E79" s="12" t="str">
-        <x:v>OSSと二種類の貢献・広告指標でスパムを抑える。</x:v>
-      </x:c>
-      <x:c r="F79" s="12" t="str">
-        <x:v>tabnews.com.br / 原文比較表ではtabnews.br</x:v>
-      </x:c>
-      <x:c r="G79" s="12" t="str">
-        <x:v>R2</x:v>
-      </x:c>
-      <x:c r="H79" s="12" t="str">
-        <x:v>https://tabnews.com.br/</x:v>
-      </x:c>
-      <x:c r="I79" s="18" t="str">
-        <x:v>有効化済み登録アカウント</x:v>
-      </x:c>
-      <x:c r="J79" s="19" t="n">
-        <x:v>45252</x:v>
-      </x:c>
-      <x:c r="K79" s="18" t="str">
-        <x:v>件・年末時点</x:v>
-      </x:c>
-      <x:c r="L79" s="18" t="str">
-        <x:v>2024年月平均ログイン2,595人・反応参加1,038人、日平均端末UV約5,700</x:v>
-      </x:c>
-      <x:c r="M79" s="18" t="str">
-        <x:v>2024年5,700,000PV。2,100,000訪問者は日次端末UVの年内合計。</x:v>
-      </x:c>
-      <x:c r="N79" s="18" t="str">
-        <x:v>登録数2024年末、活動・PV2024年実績</x:v>
-      </x:c>
-      <x:c r="O79" s="18" t="str">
-        <x:v>運営側の公開集計・歴史値</x:v>
-      </x:c>
-      <x:c r="P79" s="18" t="str">
-        <x:v>https://www.tabnews.com.br/FelipeBarso/tabnews-mais-de-2m-de-visitantes-e-5m-de-visualizacoes-em-2024</x:v>
-      </x:c>
-      <x:c r="Q79" s="18" t="str">
-        <x:v>人数なし／100 TabCashは通貨制度</x:v>
-      </x:c>
-      <x:c r="R79" s="18" t="str">
-        <x:v>有効化済み登録（cadastro ativo）はアクティブ利用の意味ではない。年間訪問者合計は年次の異なる人の数ではないと原文が明記。</x:v>
-      </x:c>
-      <x:c r="S79" s="20" t="d">
-        <x:v>2026-10-21T00:00:00.000Z</x:v>
-      </x:c>
+      <x:c r="A79"/>
+      <x:c r="B79"/>
+      <x:c r="C79"/>
+      <x:c r="D79"/>
+      <x:c r="E79"/>
+      <x:c r="F79"/>
+      <x:c r="G79"/>
+      <x:c r="H79"/>
+      <x:c r="I79"/>
+      <x:c r="J79"/>
+      <x:c r="K79"/>
+      <x:c r="L79"/>
+      <x:c r="M79"/>
+      <x:c r="N79"/>
+      <x:c r="O79"/>
+      <x:c r="P79"/>
+      <x:c r="Q79"/>
+      <x:c r="R79"/>
+      <x:c r="S79"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7fe713255e1d4b01"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rca85316ca1cc4074"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -6815,7 +6787,7 @@
         <x:v>構造・対象</x:v>
       </x:c>
       <x:c r="E107" s="12" t="str">
-        <x:v>プログラマー、独立開発者、デザイナー向けノード型掲示板。言語、DB、OS、ハードウェア、キャリア等に分類。分享創造ノードはアクセス・インストール・実行できるツール、OSS、技術製品の公開先で無料露出を得る。初期1,000人の利用者獲得チャネルとしてEleduckと共に位置付け。</x:v>
+        <x:v>プログラマー、独立開発者、デザイナー向けノード型掲示板。言語、DB、OS、ハードウェア、キャリア等に分類。分享創造ノードはアクセス・インストール・実行できるツール、OSS、技術製品の公開先で無料露出を得る。初期1,000人の利用者獲得チャネルとして位置付け。</x:v>
       </x:c>
       <x:c r="F107" s="12" t="str">
         <x:v>R2</x:v>
@@ -6863,19 +6835,19 @@
     </x:row>
     <x:row r="110" ht="44" customHeight="1">
       <x:c r="A110" s="11" t="str">
-        <x:v>P62</x:v>
+        <x:v>P63</x:v>
       </x:c>
       <x:c r="B110" s="11" t="str">
-        <x:v>電鴨社区</x:v>
+        <x:v>CSDN</x:v>
       </x:c>
       <x:c r="C110" s="11" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D110" s="11" t="str">
-        <x:v>対象・出自</x:v>
+        <x:v>対象・用途</x:v>
       </x:c>
       <x:c r="E110" s="11" t="str">
-        <x:v>中国最初期のリモートワークコミュニティ。フリーランス、リモート、外注、副業・兼業等の働き方を求めるインターネット実務者・独立開発者が集まる。</x:v>
+        <x:v>中国語圏の広いソフトウェア開発者・IT実務者向け。大量のブログ・コミュニティ記事のアーカイブ。製品公開や即時フィードバックを担うV2EXとは役割が異なると説明。</x:v>
       </x:c>
       <x:c r="F110" s="11" t="str">
         <x:v>R2</x:v>
@@ -6883,19 +6855,19 @@
     </x:row>
     <x:row r="111" ht="44" customHeight="1">
       <x:c r="A111" s="12" t="str">
-        <x:v>P62</x:v>
+        <x:v>P64</x:v>
       </x:c>
       <x:c r="B111" s="12" t="str">
-        <x:v>電鴨社区</x:v>
+        <x:v>Developpez.com</x:v>
       </x:c>
       <x:c r="C111" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D111" s="12" t="str">
-        <x:v>機能・用途</x:v>
+        <x:v>規模・沿革</x:v>
       </x:c>
       <x:c r="E111" s="12" t="str">
-        <x:v>価値あるトピック議論、案件・人材マッチング、独立製品の公開が柱。常時投稿し相互試用と反応を得る。初期1,000人の利用者獲得、外注・兼業の機会共有、初期ユーザー基盤形成に利用。</x:v>
+        <x:v>1999年創設。月間最大400万UU、日次フォーラム投稿5,000件以上、講座・記事14,000件以上、FAQ100以上。Delphi/C++/Java/RDBMS/CORBAから出発。2001年求人、2003年チャット、2004年ブログ、2005年無料ダウンロード雑誌を追加。</x:v>
       </x:c>
       <x:c r="F111" s="12" t="str">
         <x:v>R2</x:v>
@@ -6903,19 +6875,19 @@
     </x:row>
     <x:row r="112" ht="44" customHeight="1">
       <x:c r="A112" s="11" t="str">
-        <x:v>P63</x:v>
+        <x:v>P64</x:v>
       </x:c>
       <x:c r="B112" s="11" t="str">
-        <x:v>CSDN</x:v>
+        <x:v>Developpez.com</x:v>
       </x:c>
       <x:c r="C112" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D112" s="11" t="str">
-        <x:v>対象・用途</x:v>
+        <x:v>運営・活動</x:v>
       </x:c>
       <x:c r="E112" s="11" t="str">
-        <x:v>中国語圏の広いソフトウェア開発者・IT実務者向け。大量のブログ・コミュニティ記事のアーカイブ。製品公開や即時フィードバックを担うV2EX/Eleduckとは役割が異なると説明。</x:v>
+        <x:v>IT専門家、開発者、DBA、学生向け。専用サーバー群、ボランティア編集者・モデレーター。半年ごとに執筆・校閲・運営・ニュース投稿者を表彰するPalmarès。週末オンラインゲーム共同開発イベントも開催。国内採用・キャリアと接続。</x:v>
       </x:c>
       <x:c r="F112" s="11" t="str">
         <x:v>R2</x:v>
@@ -6929,13 +6901,13 @@
         <x:v>Developpez.com</x:v>
       </x:c>
       <x:c r="C113" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D113" s="12" t="str">
-        <x:v>規模・沿革</x:v>
+        <x:v>2026年10月の話題</x:v>
       </x:c>
       <x:c r="E113" s="12" t="str">
-        <x:v>1999年創設。月間最大400万UU、日次フォーラム投稿5,000件以上、講座・記事14,000件以上、FAQ100以上。Delphi/C++/Java/RDBMS/CORBAから出発。2001年求人、2003年チャット、2004年ブログ、2005年無料ダウンロード雑誌を追加。</x:v>
+        <x:v>会員ブログ/forums/blogs/ではApple Siliconでの音楽生成AIのメモリ帯域ボトルネック、MCP解説。フォーラムではPostgreSQL19、KMP0.13、Lazarus5.0、Web Worker、VBA/VB6等を議論。原文の技術名・版数をそのまま保持。</x:v>
       </x:c>
       <x:c r="F113" s="12" t="str">
         <x:v>R2</x:v>
@@ -6949,13 +6921,13 @@
         <x:v>Developpez.com</x:v>
       </x:c>
       <x:c r="C114" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D114" s="11" t="str">
-        <x:v>運営・活動</x:v>
+        <x:v>構造変化</x:v>
       </x:c>
       <x:c r="E114" s="11" t="str">
-        <x:v>IT専門家、開発者、DBA、学生向け。専用サーバー群、ボランティア編集者・モデレーター。半年ごとに執筆・校閲・運営・ニュース投稿者を表彰するPalmarès。週末オンラインゲーム共同開発イベントも開催。国内採用・キャリアと接続。</x:v>
+        <x:v>ActualitésニュースやPolitiqueでAI投資の減損リスク、EUのSNS年齢制限、国内政治等が1記事200〜600件以上のコメントを集める。開発以外の時事・政治が流入の相当部分を占め、コミュニティ変質の指摘もあると記載。</x:v>
       </x:c>
       <x:c r="F114" s="11" t="str">
         <x:v>R2</x:v>
@@ -6963,19 +6935,19 @@
     </x:row>
     <x:row r="115" ht="44" customHeight="1">
       <x:c r="A115" s="12" t="str">
-        <x:v>P64</x:v>
+        <x:v>P65</x:v>
       </x:c>
       <x:c r="B115" s="12" t="str">
-        <x:v>Developpez.com</x:v>
+        <x:v>Zeste de Savoir</x:v>
       </x:c>
       <x:c r="C115" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D115" s="12" t="str">
-        <x:v>2026年10月の話題</x:v>
+        <x:v>沿革・運営</x:v>
       </x:c>
       <x:c r="E115" s="12" t="str">
-        <x:v>会員ブログ/forums/blogs/ではApple Siliconでの音楽生成AIのメモリ帯域ボトルネック、MCP解説。フォーラムではPostgreSQL19、KMP0.13、Lazarus5.0、Web Worker、VBA/VB6等を議論。原文の技術名・版数をそのまま保持。</x:v>
+        <x:v>2014年4月、フランス1901年法の非営利協会として設立。Site du ZéroのOpenClassroomsへの改称・商業教育化に反発して辞任した元ボランティアや貢献者が設立。</x:v>
       </x:c>
       <x:c r="F115" s="12" t="str">
         <x:v>R2</x:v>
@@ -6983,19 +6955,19 @@
     </x:row>
     <x:row r="116" ht="44" customHeight="1">
       <x:c r="A116" s="11" t="str">
-        <x:v>P64</x:v>
+        <x:v>P65</x:v>
       </x:c>
       <x:c r="B116" s="11" t="str">
-        <x:v>Developpez.com</x:v>
+        <x:v>Zeste de Savoir</x:v>
       </x:c>
       <x:c r="C116" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D116" s="11" t="str">
-        <x:v>構造変化</x:v>
+        <x:v>対象・機能</x:v>
       </x:c>
       <x:c r="E116" s="11" t="str">
-        <x:v>ActualitésニュースやPolitiqueでAI投資の減損リスク、EUのSNS年齢制限、国内政治等が1記事200〜600件以上のコメントを集める。開発以外の時事・政治が流入の相当部分を占め、コミュニティ変質の指摘もあると記載。</x:v>
+        <x:v>フランス語圏の学習者・エンジニア向け。コミュニティが執筆・査読するオープンな情報科学チュートリアル・技術記事。非営利の知識共有を継承。</x:v>
       </x:c>
       <x:c r="F116" s="11" t="str">
         <x:v>R2</x:v>
@@ -7003,39 +6975,39 @@
     </x:row>
     <x:row r="117" ht="44" customHeight="1">
       <x:c r="A117" s="12" t="str">
-        <x:v>P65</x:v>
+        <x:v>P66</x:v>
       </x:c>
       <x:c r="B117" s="12" t="str">
-        <x:v>Zeste de Savoir</x:v>
+        <x:v>OpenClassrooms</x:v>
       </x:c>
       <x:c r="C117" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D117" s="12" t="str">
-        <x:v>沿革・運営</x:v>
+        <x:v>沿革・機能</x:v>
       </x:c>
       <x:c r="E117" s="12" t="str">
-        <x:v>2014年4月、フランス1901年法の非営利協会として設立。Site du ZéroのOpenClassroomsへの改称・商業教育化に反発して辞任した元ボランティアや貢献者が設立。</x:v>
+        <x:v>旧Site du Zéroの初心者向けチュートリアル共有が改称後、国際展開、オンライン学位、給与を得て学ぶalternance、企業採用へ転換。メンター付き有償・公的資金支援のキャリア教育で理論20%・実践80%と記載。Zeste de Savoir設立の背景。</x:v>
       </x:c>
       <x:c r="F117" s="12" t="str">
         <x:v>R2</x:v>
       </x:c>
     </x:row>
-    <x:row r="118" ht="44" customHeight="1">
+    <x:row r="118" ht="60" customHeight="1">
       <x:c r="A118" s="11" t="str">
-        <x:v>P65</x:v>
+        <x:v>P67</x:v>
       </x:c>
       <x:c r="B118" s="11" t="str">
-        <x:v>Zeste de Savoir</x:v>
+        <x:v>Les Pépites Tech</x:v>
       </x:c>
       <x:c r="C118" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D118" s="11" t="str">
-        <x:v>対象・機能</x:v>
+        <x:v>規模・沿革</x:v>
       </x:c>
       <x:c r="E118" s="11" t="str">
-        <x:v>フランス語圏の学習者・エンジニア向け。コミュニティが執筆・査読するオープンな情報科学チュートリアル・技術記事。非営利の知識共有を継承。</x:v>
+        <x:v>2015年創設、4,237社以上を収録。La French Techの公式パートナーディレクトリとの説明。国内13のFrench Tech首都と世界38コミュニティを横断。例はGrand Paris、Lille、Brest Bretagne Ouest、Aix-Marseille Région Sud、Pays Basque、海外はバルセロナ・アルジェ等。</x:v>
       </x:c>
       <x:c r="F118" s="11" t="str">
         <x:v>R2</x:v>
@@ -7043,25 +7015,25 @@
     </x:row>
     <x:row r="119" ht="44" customHeight="1">
       <x:c r="A119" s="12" t="str">
-        <x:v>P66</x:v>
+        <x:v>P67</x:v>
       </x:c>
       <x:c r="B119" s="12" t="str">
-        <x:v>OpenClassrooms</x:v>
+        <x:v>Les Pépites Tech</x:v>
       </x:c>
       <x:c r="C119" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D119" s="12" t="str">
-        <x:v>沿革・機能</x:v>
+        <x:v>公開・評価</x:v>
       </x:c>
       <x:c r="E119" s="12" t="str">
-        <x:v>旧Site du Zéroの初心者向けチュートリアル共有が改称後、国際展開、オンライン学位、給与を得て学ぶalternance、企業採用へ転換。メンター付き有償・公的資金支援のキャリア教育で理論20%・実践80%と記載。Zeste de Savoir設立の背景。</x:v>
+        <x:v>Google/LinkedIn/X（旧Twitter）ログイン、メンバーのアップボート。週間Best of de la semaine、月間、歴代のランキング。地域拠点・業種別コレクションで分類。スタートアップ・SaaS・AI開発者向け。</x:v>
       </x:c>
       <x:c r="F119" s="12" t="str">
         <x:v>R2</x:v>
       </x:c>
     </x:row>
-    <x:row r="120" ht="60" customHeight="1">
+    <x:row r="120" ht="44" customHeight="1">
       <x:c r="A120" s="11" t="str">
         <x:v>P67</x:v>
       </x:c>
@@ -7069,13 +7041,13 @@
         <x:v>Les Pépites Tech</x:v>
       </x:c>
       <x:c r="C120" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D120" s="11" t="str">
-        <x:v>規模・沿革</x:v>
+        <x:v>製品群・地域性</x:v>
       </x:c>
       <x:c r="E120" s="11" t="str">
-        <x:v>2015年創設、4,237社以上を収録。La French Techの公式パートナーディレクトリとの説明。国内13のFrench Tech首都と世界38コミュニティを横断。例はGrand Paris、Lille、Brest Bretagne Ouest、Aix-Marseille Région Sud、Pays Basque、海外はバルセロナ・アルジェ等。</x:v>
+        <x:v>主権型・省資源AI、AI Act/RGPD/NIS2/DORA/SecNumCloud/ISO27001対応のRegTech・SaaS、医療・自由業の社会保障費管理、建設職人やTPE/PMEの音声見積・電子請求書を支えるAIエージェントが集積すると記載。Sovkern等8件は関連事例表。</x:v>
       </x:c>
       <x:c r="F120" s="11" t="str">
         <x:v>R2</x:v>
@@ -7089,13 +7061,13 @@
         <x:v>Les Pépites Tech</x:v>
       </x:c>
       <x:c r="C121" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D121" s="12" t="str">
-        <x:v>公開・評価</x:v>
+        <x:v>活用</x:v>
       </x:c>
       <x:c r="E121" s="12" t="str">
-        <x:v>Google/LinkedIn/X（旧Twitter）ログイン、メンバーのアップボート。週間Best of de la semaine、月間、歴代のランキング。地域拠点・業種別コレクションで分類。スタートアップ・SaaS・AI開発者向け。</x:v>
+        <x:v>現地の制度・文化・商慣習と接続したB2B製品の発見・公開先。活用時はRGPD/AI Act等への適合性や具体的技術スタックを明示する提案。</x:v>
       </x:c>
       <x:c r="F121" s="12" t="str">
         <x:v>R2</x:v>
@@ -7103,19 +7075,19 @@
     </x:row>
     <x:row r="122" ht="44" customHeight="1">
       <x:c r="A122" s="11" t="str">
-        <x:v>P67</x:v>
+        <x:v>P68</x:v>
       </x:c>
       <x:c r="B122" s="11" t="str">
-        <x:v>Les Pépites Tech</x:v>
+        <x:v>WeLoveDevs.com</x:v>
       </x:c>
       <x:c r="C122" s="11" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D122" s="11" t="str">
-        <x:v>製品群・地域性</x:v>
+        <x:v>規模・機能</x:v>
       </x:c>
       <x:c r="E122" s="11" t="str">
-        <x:v>主権型・省資源AI、AI Act/RGPD/NIS2/DORA/SecNumCloud/ISO27001対応のRegTech・SaaS、医療・自由業の社会保障費管理、建設職人やTPE/PMEの音声見積・電子請求書を支えるAIエージェントが集積すると記載。Sovkern等8件は関連事例表。</x:v>
+        <x:v>月間技術訪問者4万人以上、参画企業2,500〜3,000社以上。Web開発者、データ科学者、DevOps向け。ポートフォリオと給与・リモート条件を明示した求人マッチング。国内採用・キャリア形成と接続。</x:v>
       </x:c>
       <x:c r="F122" s="11" t="str">
         <x:v>R2</x:v>
@@ -7123,19 +7095,19 @@
     </x:row>
     <x:row r="123" ht="44" customHeight="1">
       <x:c r="A123" s="12" t="str">
-        <x:v>P67</x:v>
+        <x:v>P68</x:v>
       </x:c>
       <x:c r="B123" s="12" t="str">
-        <x:v>Les Pépites Tech</x:v>
+        <x:v>WeLoveDevs.com</x:v>
       </x:c>
       <x:c r="C123" s="12" t="n">
-        <x:v>4</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D123" s="12" t="str">
-        <x:v>活用</x:v>
+        <x:v>関係</x:v>
       </x:c>
       <x:c r="E123" s="12" t="str">
-        <x:v>現地の制度・文化・商慣習と接続したB2B製品の発見・公開先。活用時はRGPD/AI Act等への適合性や具体的技術スタックを明示する提案。</x:v>
+        <x:v>傘下のCodersTestsは別行。原文のWeLoveDevs / CodersTests共同行にある開発者3万人以上・QCM100以上は、本文でCodersTests側に対応付くため分離。</x:v>
       </x:c>
       <x:c r="F123" s="12" t="str">
         <x:v>R2</x:v>
@@ -7143,10 +7115,10 @@
     </x:row>
     <x:row r="124" ht="44" customHeight="1">
       <x:c r="A124" s="11" t="str">
-        <x:v>P68</x:v>
+        <x:v>P69</x:v>
       </x:c>
       <x:c r="B124" s="11" t="str">
-        <x:v>WeLoveDevs.com</x:v>
+        <x:v>CodersTests</x:v>
       </x:c>
       <x:c r="C124" s="11" t="n">
         <x:v>1</x:v>
@@ -7155,7 +7127,7 @@
         <x:v>規模・機能</x:v>
       </x:c>
       <x:c r="E124" s="11" t="str">
-        <x:v>月間技術訪問者4万人以上、参画企業2,500〜3,000社以上。Web開発者、データ科学者、DevOps向け。ポートフォリオと給与・リモート条件を明示した求人マッチング。国内採用・キャリア形成と接続。</x:v>
+        <x:v>WeLoveDevs傘下、開発者登録3万人以上、専門家作成の技術QCM100種類以上。React/Laravel/Tailwind/セキュリティ等でメダルを獲得し、ポートフォリオと求人マッチングにつながる。</x:v>
       </x:c>
       <x:c r="F124" s="11" t="str">
         <x:v>R2</x:v>
@@ -7163,19 +7135,19 @@
     </x:row>
     <x:row r="125" ht="44" customHeight="1">
       <x:c r="A125" s="12" t="str">
-        <x:v>P68</x:v>
+        <x:v>P70</x:v>
       </x:c>
       <x:c r="B125" s="12" t="str">
-        <x:v>WeLoveDevs.com</x:v>
+        <x:v>Velog</x:v>
       </x:c>
       <x:c r="C125" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D125" s="12" t="str">
-        <x:v>関係</x:v>
+        <x:v>運営・機能</x:v>
       </x:c>
       <x:c r="E125" s="12" t="str">
-        <x:v>傘下のCodersTestsは別行。原文のWeLoveDevs / CodersTests共同行にある開発者3万人以上・QCM100以上は、本文でCodersTests側に対応付くため分離。</x:v>
+        <x:v>velopertが開発・公開したOSS起源のブログ基盤。韓国語のみをサポートすると原文は説明。余計な装飾を排したMarkdownエディタとシンタックスハイライト。</x:v>
       </x:c>
       <x:c r="F125" s="12" t="str">
         <x:v>R2</x:v>
@@ -7183,19 +7155,19 @@
     </x:row>
     <x:row r="126" ht="44" customHeight="1">
       <x:c r="A126" s="11" t="str">
-        <x:v>P69</x:v>
+        <x:v>P70</x:v>
       </x:c>
       <x:c r="B126" s="11" t="str">
-        <x:v>CodersTests</x:v>
+        <x:v>Velog</x:v>
       </x:c>
       <x:c r="C126" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D126" s="11" t="str">
-        <x:v>規模・機能</x:v>
+        <x:v>用途</x:v>
       </x:c>
       <x:c r="E126" s="11" t="str">
-        <x:v>WeLoveDevs傘下、開発者登録3万人以上、専門家作成の技術QCM100種類以上。React/Laravel/Tailwind/セキュリティ等でメダルを獲得し、ポートフォリオと求人マッチングにつながる。</x:v>
+        <x:v>学習記録、アルゴリズム解説、SAP等の認定試験対策、フレームワーク実装知見を蓄積。韓国の技術ブログ標準基盤、OKKY/Disquietとは役割分担。</x:v>
       </x:c>
       <x:c r="F126" s="11" t="str">
         <x:v>R2</x:v>
@@ -7203,19 +7175,19 @@
     </x:row>
     <x:row r="127" ht="44" customHeight="1">
       <x:c r="A127" s="12" t="str">
-        <x:v>P70</x:v>
+        <x:v>P71</x:v>
       </x:c>
       <x:c r="B127" s="12" t="str">
-        <x:v>Velog</x:v>
+        <x:v>Disquiet</x:v>
       </x:c>
       <x:c r="C127" s="12" t="n">
         <x:v>1</x:v>
       </x:c>
       <x:c r="D127" s="12" t="str">
-        <x:v>運営・機能</x:v>
+        <x:v>規模・目的</x:v>
       </x:c>
       <x:c r="E127" s="12" t="str">
-        <x:v>velopertが開発・公開したOSS起源のブログ基盤。韓国語のみをサポートすると原文は説明。余計な装飾を排したMarkdownエディタとシンタックスハイライト。</x:v>
+        <x:v>月間新規製品200件以上は2023年基準。個人メイカー、一人創業者、ITチーム、VC向け。KBインベストメント等の投資家からの接触、共同創業者や採用候補の発掘、初期顧客とフィードバック獲得。</x:v>
       </x:c>
       <x:c r="F127" s="12" t="str">
         <x:v>R2</x:v>
@@ -7223,19 +7195,19 @@
     </x:row>
     <x:row r="128" ht="44" customHeight="1">
       <x:c r="A128" s="11" t="str">
-        <x:v>P70</x:v>
+        <x:v>P71</x:v>
       </x:c>
       <x:c r="B128" s="11" t="str">
-        <x:v>Velog</x:v>
+        <x:v>Disquiet</x:v>
       </x:c>
       <x:c r="C128" s="11" t="n">
         <x:v>2</x:v>
       </x:c>
       <x:c r="D128" s="11" t="str">
-        <x:v>用途</x:v>
+        <x:v>機能・評価</x:v>
       </x:c>
       <x:c r="E128" s="11" t="str">
-        <x:v>学習記録、アルゴリズム解説、SAP等の認定試験対策、フレームワーク実装知見を蓄積。韓国の技術ブログ標準基盤、OKKY/Disquietとは役割分担。</x:v>
+        <x:v>常時製品登録とメイカーログ更新。開発記録を製品へ直結させ、プロフィールに開発中製品と関心トピックを表示。一回限りのローンチで埋もれる問題を軽減し、継続露出を得る。UI改修理由や配送先変更ロジック等の意思決定も共有。</x:v>
       </x:c>
       <x:c r="F128" s="11" t="str">
         <x:v>R2</x:v>
@@ -7249,13 +7221,13 @@
         <x:v>Disquiet</x:v>
       </x:c>
       <x:c r="C129" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D129" s="12" t="str">
-        <x:v>規模・目的</x:v>
+        <x:v>事例・組織文化</x:v>
       </x:c>
       <x:c r="E129" s="12" t="str">
-        <x:v>月間新規製品200件以上は2023年基準。個人メイカー、一人創業者、ITチーム、VC向け。KBインベストメント等の投資家からの接触、共同創業者や採用候補の発掘、初期顧客とフィードバック獲得。</x:v>
+        <x:v>Wonderday、SIGNUM HQ、OfficialMail、Zaemit AI、Oriberを例示。詳細は関連事例表。自社開発では企画者から仕様・デザインを受け取る方式より、エンジニア自身がAARRRの観点で課題定義から実装・顧客フィードバックまで主導すると説明。</x:v>
       </x:c>
       <x:c r="F129" s="12" t="str">
         <x:v>R2</x:v>
@@ -7263,19 +7235,19 @@
     </x:row>
     <x:row r="130" ht="44" customHeight="1">
       <x:c r="A130" s="11" t="str">
-        <x:v>P71</x:v>
+        <x:v>P72</x:v>
       </x:c>
       <x:c r="B130" s="11" t="str">
-        <x:v>Disquiet</x:v>
+        <x:v>OKKY</x:v>
       </x:c>
       <x:c r="C130" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D130" s="11" t="str">
-        <x:v>機能・評価</x:v>
+        <x:v>用途</x:v>
       </x:c>
       <x:c r="E130" s="11" t="str">
-        <x:v>常時製品登録とメイカーログ更新。開発記録を製品へ直結させ、プロフィールに開発中製品と関心トピックを表示。一回限りのローンチで埋もれる問題を軽減し、継続露出を得る。UI改修理由や配送先変更ロジック等の意思決定も共有。</x:v>
+        <x:v>韓国のソフトウェアエンジニア全般。技術Q&amp;A、実務経験、キャリア議論。伝統的なQ&amp;A・キャリア掲示板でVelog/Disquietと役割を分担。</x:v>
       </x:c>
       <x:c r="F130" s="11" t="str">
         <x:v>R2</x:v>
@@ -7283,19 +7255,19 @@
     </x:row>
     <x:row r="131" ht="44" customHeight="1">
       <x:c r="A131" s="12" t="str">
-        <x:v>P71</x:v>
+        <x:v>P73</x:v>
       </x:c>
       <x:c r="B131" s="12" t="str">
-        <x:v>Disquiet</x:v>
+        <x:v>Habr</x:v>
       </x:c>
       <x:c r="C131" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D131" s="12" t="str">
-        <x:v>事例・組織文化</x:v>
+        <x:v>対象・公開条件</x:v>
       </x:c>
       <x:c r="E131" s="12" t="str">
-        <x:v>Wonderday、SIGNUM HQ、OfficialMail、Zaemit AI、Oriberを例示。詳細は関連事例表。自社開発では企画者から仕様・デザインを受け取る方式より、エンジニア自身がAARRRの観点で課題定義から実装・顧客フィードバックまで主導すると説明。</x:v>
+        <x:v>ロシア・旧ソ連圏のシニア開発者、IT専門家、技術企業。新規ユーザーはサンドボックス（песочница）に記事を出し、既存会員・モデレーターから招待と承認を得る。</x:v>
       </x:c>
       <x:c r="F131" s="12" t="str">
         <x:v>R2</x:v>
@@ -7303,19 +7275,19 @@
     </x:row>
     <x:row r="132" ht="44" customHeight="1">
       <x:c r="A132" s="11" t="str">
-        <x:v>P72</x:v>
+        <x:v>P73</x:v>
       </x:c>
       <x:c r="B132" s="11" t="str">
-        <x:v>OKKY</x:v>
+        <x:v>Habr</x:v>
       </x:c>
       <x:c r="C132" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D132" s="11" t="str">
-        <x:v>用途</x:v>
+        <x:v>評価制度</x:v>
       </x:c>
       <x:c r="E132" s="11" t="str">
-        <x:v>韓国のソフトウェアエンジニア全般。技術Q&amp;A、実務経験、キャリア議論。伝統的なQ&amp;A・キャリア掲示板でVelog/Disquietと役割を分担。</x:v>
+        <x:v>個人へのカルマと記事・コメントへのレーティングを分離。記事/コメントへの投票は公開後30日間で変更不可。個人カルマへの投票は期限なし、いつでも変更可能。</x:v>
       </x:c>
       <x:c r="F132" s="11" t="str">
         <x:v>R2</x:v>
@@ -7329,13 +7301,13 @@
         <x:v>Habr</x:v>
       </x:c>
       <x:c r="C133" s="12" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D133" s="12" t="str">
-        <x:v>対象・公開条件</x:v>
+        <x:v>著者報奨参加条件</x:v>
       </x:c>
       <x:c r="E133" s="12" t="str">
-        <x:v>ロシア・旧ソ連圏のシニア開発者、IT専門家、技術企業。新規ユーザーはサンドボックス（песочница）に記事を出し、既存会員・モデレーターから招待と承認を得る。</x:v>
+        <x:v>ППА（著者奨励プログラム）は、アカウント3年以上かつカルマ+50超、またはレーティング+50超の記事10本以上かつカルマ+50超が条件。</x:v>
       </x:c>
       <x:c r="F133" s="12" t="str">
         <x:v>R2</x:v>
@@ -7349,13 +7321,13 @@
         <x:v>Habr</x:v>
       </x:c>
       <x:c r="C134" s="11" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D134" s="11" t="str">
-        <x:v>評価制度</x:v>
+        <x:v>報酬</x:v>
       </x:c>
       <x:c r="E134" s="11" t="str">
-        <x:v>個人へのカルマと記事・コメントへのレーティングを分離。記事/コメントへの投票は公開後30日間で変更不可。個人カルマへの投票は期限なし、いつでも変更可能。</x:v>
+        <x:v>記事レーティング+30で3,000ルーブル、+50で5,000ルーブル、閾値を超える1点につき10ルーブルを加算。翻訳カテゴリは最終報酬50%。翻訳で+134なら通常5,840ルーブルの半額2,920ルーブルという例。</x:v>
       </x:c>
       <x:c r="F134" s="11" t="str">
         <x:v>R2</x:v>
@@ -7369,13 +7341,13 @@
         <x:v>Habr</x:v>
       </x:c>
       <x:c r="C135" s="12" t="n">
-        <x:v>3</x:v>
+        <x:v>5</x:v>
       </x:c>
       <x:c r="D135" s="12" t="str">
-        <x:v>著者報奨参加条件</x:v>
+        <x:v>出金・狙い</x:v>
       </x:c>
       <x:c r="E135" s="12" t="str">
-        <x:v>ППА（著者奨励プログラム）は、アカウント3年以上かつカルマ+50超、またはレーティング+50超の記事10本以上かつカルマ+50超が条件。</x:v>
+        <x:v>最低出金3,000ルーブル。自動出金設定後、翌月初めに担当者が連絡し銀行カード等へ送金。翻訳よりオリジナル一次技術情報を優遇する設計。現地発信ではサンドボックス突破を提案。</x:v>
       </x:c>
       <x:c r="F135" s="12" t="str">
         <x:v>R2</x:v>
@@ -7383,19 +7355,19 @@
     </x:row>
     <x:row r="136" ht="44" customHeight="1">
       <x:c r="A136" s="11" t="str">
-        <x:v>P73</x:v>
+        <x:v>P74</x:v>
       </x:c>
       <x:c r="B136" s="11" t="str">
-        <x:v>Habr</x:v>
+        <x:v>TabNews</x:v>
       </x:c>
       <x:c r="C136" s="11" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
       <x:c r="D136" s="11" t="str">
-        <x:v>報酬</x:v>
+        <x:v>運営・開発</x:v>
       </x:c>
       <x:c r="E136" s="11" t="str">
-        <x:v>記事レーティング+30で3,000ルーブル、+50で5,000ルーブル、閾値を超える1点につき10ルーブルを加算。翻訳カテゴリは最終報酬50%。翻訳で+134なら通常5,840ルーブルの半額2,920ルーブルという例。</x:v>
+        <x:v>Filipe Deschampsらが主導しFabio Akitaも議論に関与。GitHub上でサイト自体をOSS開発し、利用者がセキュリティ改善・SEO最適化に貢献。</x:v>
       </x:c>
       <x:c r="F136" s="11" t="str">
         <x:v>R2</x:v>
@@ -7403,19 +7375,19 @@
     </x:row>
     <x:row r="137" ht="44" customHeight="1">
       <x:c r="A137" s="12" t="str">
-        <x:v>P73</x:v>
+        <x:v>P74</x:v>
       </x:c>
       <x:c r="B137" s="12" t="str">
-        <x:v>Habr</x:v>
+        <x:v>TabNews</x:v>
       </x:c>
       <x:c r="C137" s="12" t="n">
-        <x:v>5</x:v>
+        <x:v>2</x:v>
       </x:c>
       <x:c r="D137" s="12" t="str">
-        <x:v>出金・狙い</x:v>
+        <x:v>課題・評価</x:v>
       </x:c>
       <x:c r="E137" s="12" t="str">
-        <x:v>最低出金3,000ルーブル。自動出金設定後、翌月初めに担当者が連絡し銀行カード等へ送金。翻訳よりオリジナル一次技術情報を優遇する設計。現地発信ではサンドボックス突破を提案。</x:v>
+        <x:v>SaaS宣伝の氾濫とモデレーション負荷への対策として、内部通貨TabCoinsとTabCashを分離。TabCoinsは有益な記事・コメントの評価による貢献・評判指標で、低評価で失う。</x:v>
       </x:c>
       <x:c r="F137" s="12" t="str">
         <x:v>R2</x:v>
@@ -7429,13 +7401,13 @@
         <x:v>TabNews</x:v>
       </x:c>
       <x:c r="C138" s="11" t="n">
-        <x:v>1</x:v>
+        <x:v>3</x:v>
       </x:c>
       <x:c r="D138" s="11" t="str">
-        <x:v>運営・開発</x:v>
+        <x:v>広告・制御</x:v>
       </x:c>
       <x:c r="E138" s="11" t="str">
-        <x:v>Filipe Deschampsらが主導しFabio Akitaも議論に関与。GitHub上でサイト自体をOSS開発し、利用者がセキュリティ改善・SEO最適化に貢献。</x:v>
+        <x:v>スポンサー投稿はTabCoinsを付与せず、TabCashを消費する設計と原文は説明。読者が単なる広告と判定するフィードバックや、100 TabCash以上の保有者のシステム利用枠を挙げる。経済コストと露出制御でSEO価値・議論を保護。</x:v>
       </x:c>
       <x:c r="F138" s="11" t="str">
         <x:v>R2</x:v>
@@ -7449,62 +7421,38 @@
         <x:v>TabNews</x:v>
       </x:c>
       <x:c r="C139" s="12" t="n">
-        <x:v>2</x:v>
+        <x:v>4</x:v>
       </x:c>
       <x:c r="D139" s="12" t="str">
-        <x:v>課題・評価</x:v>
+        <x:v>URL表記差</x:v>
       </x:c>
       <x:c r="E139" s="12" t="str">
-        <x:v>SaaS宣伝の氾濫とモデレーション負荷への対策として、内部通貨TabCoinsとTabCashを分離。TabCoinsは有益な記事・コメントの評価による貢献・評判指標で、低評価で失う。</x:v>
+        <x:v>比較表にtabnews.br、本文にtabnews.com.brの両表記。原文の差を記録し、URL欄は本文の完全表記を採用。転記を越える公式仕様・通貨制度の正確性検証は行っていない。</x:v>
       </x:c>
       <x:c r="F139" s="12" t="str">
         <x:v>R2</x:v>
       </x:c>
     </x:row>
     <x:row r="140" ht="44" customHeight="1">
-      <x:c r="A140" s="11" t="str">
-        <x:v>P74</x:v>
-      </x:c>
-      <x:c r="B140" s="11" t="str">
-        <x:v>TabNews</x:v>
-      </x:c>
-      <x:c r="C140" s="11" t="n">
-        <x:v>3</x:v>
-      </x:c>
-      <x:c r="D140" s="11" t="str">
-        <x:v>広告・制御</x:v>
-      </x:c>
-      <x:c r="E140" s="11" t="str">
-        <x:v>スポンサー投稿はTabCoinsを付与せず、TabCashを消費する設計と原文は説明。読者が単なる広告と判定するフィードバックや、100 TabCash以上の保有者のシステム利用枠を挙げる。経済コストと露出制御でSEO価値・議論を保護。</x:v>
-      </x:c>
-      <x:c r="F140" s="11" t="str">
-        <x:v>R2</x:v>
-      </x:c>
+      <x:c r="A140"/>
+      <x:c r="B140"/>
+      <x:c r="C140"/>
+      <x:c r="D140"/>
+      <x:c r="E140"/>
+      <x:c r="F140"/>
     </x:row>
     <x:row r="141" ht="44" customHeight="1">
-      <x:c r="A141" s="12" t="str">
-        <x:v>P74</x:v>
-      </x:c>
-      <x:c r="B141" s="12" t="str">
-        <x:v>TabNews</x:v>
-      </x:c>
-      <x:c r="C141" s="12" t="n">
-        <x:v>4</x:v>
-      </x:c>
-      <x:c r="D141" s="12" t="str">
-        <x:v>URL表記差</x:v>
-      </x:c>
-      <x:c r="E141" s="12" t="str">
-        <x:v>比較表にtabnews.br、本文にtabnews.com.brの両表記。原文の差を記録し、URL欄は本文の完全表記を採用。転記を越える公式仕様・通貨制度の正確性検証は行っていない。</x:v>
-      </x:c>
-      <x:c r="F141" s="12" t="str">
-        <x:v>R2</x:v>
-      </x:c>
+      <x:c r="A141"/>
+      <x:c r="B141"/>
+      <x:c r="C141"/>
+      <x:c r="D141"/>
+      <x:c r="E141"/>
+      <x:c r="F141"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re2a1c69127974834"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re8644d0258844052"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -7538,7 +7486,7 @@
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="5" t="str">
-        <x:v>製品例・基盤・連携先・比較対象の名称と、名称不明の公開基盤の事例。一覧の74項目とは登場する役割を区別。</x:v>
+        <x:v>製品例・基盤・連携先・比較対象の名称と、名称不明の公開基盤の事例。一覧の73項目とは登場する役割を区別。</x:v>
       </x:c>
       <x:c r="B3" s="1"/>
       <x:c r="C3" s="1"/>
@@ -8422,7 +8370,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R142b79dc21404420"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbda15224751345cc"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8567,7 +8515,7 @@
         <x:v>地域別の発信先</x:v>
       </x:c>
       <x:c r="C14" s="11" t="str">
-        <x:v>日本はQiitaとZenn、韓国はVelogとOKKY、フランス語圏はDeveloppez.comとZeste de Savoir、ロシア語圏はHabr。製品公開は中国V2EX/Eleduck、韓国Disquiet、フランスLes Pépites Tech/WeLoveDevs等の現地文化に合わせる提案。</x:v>
+        <x:v>日本はQiitaとZenn、韓国はVelogとOKKY、フランス語圏はDeveloppez.comとZeste de Savoir、ロシア語圏はHabr。製品公開は中国V2EX、韓国Disquiet、フランスLes Pépites Tech/WeLoveDevs等の現地文化に合わせる提案。</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="60" customHeight="1">
@@ -8584,7 +8532,7 @@
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R0c1d37c1ef504ecf"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R19c217800de148f5"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -8641,7 +8589,7 @@
         <x:v>一覧の収録数</x:v>
       </x:c>
       <x:c r="C6" s="11" t="n">
-        <x:v>74</x:v>
+        <x:v>73</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="34" customHeight="1">
@@ -8663,7 +8611,7 @@
         <x:v>詳細情報行</x:v>
       </x:c>
       <x:c r="C8" s="11" t="n">
-        <x:v>136</x:v>
+        <x:v>134</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="34" customHeight="1">
@@ -8707,7 +8655,7 @@
         <x:v>R2に登場する一覧項目</x:v>
       </x:c>
       <x:c r="C12" s="11" t="n">
-        <x:v>41</x:v>
+        <x:v>40</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="34" customHeight="1">
@@ -8718,7 +8666,7 @@
         <x:v>一覧→原文の未検出名称</x:v>
       </x:c>
       <x:c r="C13" s="12" t="str">
-        <x:v>0件。全74項目を両原文のテキストと照合。R1は59項目、R2は41項目、共通26項目。</x:v>
+        <x:v>0件。掲載対象の全73項目を両原文のテキストと照合。R1は59項目、R2は40項目、共通26項目。ユーザー指定の1項目は掲載対象から除外。</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="34" customHeight="1">
@@ -8773,7 +8721,7 @@
         <x:v>網羅性の結論</x:v>
       </x:c>
       <x:c r="C18" s="11" t="str">
-        <x:v>可読の本文・見出し・比較表・結論について抽出と照合を実施。別名・内包機能は一覧または詳細、事例・連携先は関連表に収録。空の埋め込み枠に関する限界は下記を参照。</x:v>
+        <x:v>可読の本文・見出し・比較表・結論について抽出と照合を実施。ユーザー指定の1項目を除外。残る項目の別名・内包機能は一覧または詳細、事例・連携先は関連表に収録。空の埋め込み枠に関する限界は下記を参照。</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="44" customHeight="1">
@@ -8784,7 +8732,7 @@
         <x:v>抽出範囲</x:v>
       </x:c>
       <x:c r="C19" s="12" t="str">
-        <x:v>本文・見出し・比較表・結論の全てを対象。ニュースレター、休止済みサービス、サイト内コミュニティも含む。製品・連携先・比喩だけの名前は関連事例に区分。</x:v>
+        <x:v>本文・見出し・比較表・結論の全てを対象に抽出後、ユーザー指定の1項目を除外し73項目を掲載。ニュースレター、休止済みサービス、サイト内コミュニティも含む。製品・連携先・比喩だけの名前は関連事例に区分。</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="44" customHeight="1">
@@ -8993,7 +8941,7 @@
         <x:v>対象</x:v>
       </x:c>
       <x:c r="C38" s="18" t="str">
-        <x:v>一覧の全74項目。関連製品・連携先の別表は今回の規模調査対象外。</x:v>
+        <x:v>一覧の全73項目。関連製品・連携先の別表は今回の規模調査対象外。</x:v>
       </x:c>
     </x:row>
     <x:row r="39" ht="34" customHeight="1">
@@ -9048,7 +8996,7 @@
         <x:v>具体的な代表数値を未確認</x:v>
       </x:c>
       <x:c r="C43" s="11" t="n">
-        <x:v>19</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="44" ht="44" customHeight="1">
@@ -9158,13 +9106,13 @@
         <x:v>既存内容の保存</x:v>
       </x:c>
       <x:c r="C53" s="11" t="str">
-        <x:v>既存5シートと74件のID・名称・分類等を維持。「一覧」に規模列を追加し、「レビュー・出典」の末尾へ今回のレビューを追記。</x:v>
+        <x:v>ユーザー指定の1項目を除外し、既存5シートと残る73件のID・名称・分類等を維持。「一覧」に規模列を追加し、「レビュー・出典」の末尾へ今回のレビューを追記。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rb7c25dbbf395410f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rab22781fdca84731"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>